<commit_message>
feat: implement evidence driven reconciliation engine
</commit_message>
<xml_diff>
--- a/data/demo/vn_synthetic_demo/sample_reconciliation.xlsx
+++ b/data/demo/vn_synthetic_demo/sample_reconciliation.xlsx
@@ -1541,9 +1541,10 @@
           <t>ORD00028</t>
         </is>
       </c>
-      <c r="I25">
-        <f>HYPERLINK("https://invalid")</f>
-        <v/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>=HYPERLINK("https://invalid")</t>
+        </is>
       </c>
     </row>
     <row r="26">

</xml_diff>